<commit_message>
Update date format in master template and instructions
Update date examples in the master Excel template and add a note in the instructions sheet to use dd/mm/aaaa format, ensuring backend compatibility.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4c3c9ee1-2555-449f-adab-acb7a52c5b57
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A60"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -498,207 +498,212 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v>FORMATO DE FECHAS: dd/mm/aaaa   Ejemplo: 15/01/2024</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A60"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -736,7 +741,7 @@
         <v>1234567890101</v>
       </c>
       <c r="B2" t="str">
-        <v>2024-03-01</v>
+        <v>01/03/2024</v>
       </c>
       <c r="C2" t="str">
         <v>500</v>
@@ -1169,7 +1174,7 @@
         <v>Comercio</v>
       </c>
       <c r="E2" t="str">
-        <v>2024-01-15</v>
+        <v>15/01/2024</v>
       </c>
       <c r="F2" t="str">
         <v>si</v>
@@ -1443,7 +1448,7 @@
         <v>Juan García López</v>
       </c>
       <c r="C2" t="str">
-        <v>1990-05-20</v>
+        <v>20/05/1990</v>
       </c>
       <c r="D2" t="str">
         <v>masculino</v>
@@ -1473,7 +1478,7 @@
         <v>Guatemala Ciudad</v>
       </c>
       <c r="M2" t="str">
-        <v>2024-01-15</v>
+        <v>15/01/2024</v>
       </c>
       <c r="N2" t="str">
         <v>Puesto Central</v>
@@ -1572,7 +1577,7 @@
         <v>empresa</v>
       </c>
       <c r="H2" t="str">
-        <v>2024-01-01</v>
+        <v>01/01/2024</v>
       </c>
       <c r="I2" t="str">
         <v/>

</xml_diff>

<commit_message>
Update master template to correctly handle shift data
Correct the columns in the master template's 'TURNOS' sheet and the instructions sheet to accurately reflect how shift data is processed.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4d4ffb5f-bf61-4f58-b1e1-a0bf0a0064b3
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A65"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -503,207 +503,227 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A65"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1219,14 +1239,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E5"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1237,15 +1256,12 @@
         <v>horas_trabajo</v>
       </c>
       <c r="C1" t="str">
-        <v>tipo</v>
+        <v>horas_descanso</v>
       </c>
       <c r="D1" t="str">
-        <v>hora_inicio</v>
+        <v>num_titulares</v>
       </c>
       <c r="E1" t="str">
-        <v>hora_fin</v>
-      </c>
-      <c r="F1" t="str">
         <v>descripcion</v>
       </c>
     </row>
@@ -1257,21 +1273,69 @@
         <v>8</v>
       </c>
       <c r="C2" t="str">
-        <v>diurno</v>
+        <v>16</v>
       </c>
       <c r="D2" t="str">
-        <v>07:00</v>
+        <v>2</v>
       </c>
       <c r="E2" t="str">
-        <v>15:00</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Turno normal diurno</v>
+        <v>Turno diurno 07:00 a 15:00</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Turno Nocturno 8h</v>
+      </c>
+      <c r="B3" t="str">
+        <v>8</v>
+      </c>
+      <c r="C3" t="str">
+        <v>16</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Turno nocturno 23:00 a 07:00</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Turno 12h Diurno</v>
+      </c>
+      <c r="B4" t="str">
+        <v>12</v>
+      </c>
+      <c r="C4" t="str">
+        <v>12</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Jornada 12 horas diurna 06:00 a 18:00</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Turno 24x24</v>
+      </c>
+      <c r="B5" t="str">
+        <v>24</v>
+      </c>
+      <c r="C5" t="str">
+        <v>24</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Jornada 24 horas — 07:00 a 07:00 del día siguiente</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update weapon assignment logic to assign to posts instead of employees
Modify ARMAS sheet in master template to use 'puesto_nombre' as the primary assignment field and include licensing details.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 29a1f3cc-cf38-4d6b-9fae-9b7f4aabfdff
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A65"/>
+  <dimension ref="A1:A70"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -503,227 +503,247 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
+        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A70"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1572,18 +1592,22 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:N3"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1597,25 +1621,37 @@
         <v>modelo</v>
       </c>
       <c r="D1" t="str">
+        <v>calibre</v>
+      </c>
+      <c r="E1" t="str">
         <v>serie</v>
-      </c>
-      <c r="E1" t="str">
-        <v>calibre</v>
       </c>
       <c r="F1" t="str">
         <v>estado</v>
       </c>
       <c r="G1" t="str">
-        <v>propietario</v>
+        <v>codigo</v>
       </c>
       <c r="H1" t="str">
-        <v>fecha_registro</v>
+        <v>puesto_nombre</v>
       </c>
       <c r="I1" t="str">
-        <v>notas</v>
+        <v>numero_tenencia</v>
       </c>
       <c r="J1" t="str">
-        <v>asignado_a_dpi</v>
+        <v>fecha_vencimiento_tenencia</v>
+      </c>
+      <c r="K1" t="str">
+        <v>numero_portacion</v>
+      </c>
+      <c r="L1" t="str">
+        <v>fecha_vencimiento_portacion</v>
+      </c>
+      <c r="M1" t="str">
+        <v>custodio_dpi</v>
+      </c>
+      <c r="N1" t="str">
+        <v>observaciones</v>
       </c>
     </row>
     <row r="2">
@@ -1629,30 +1665,86 @@
         <v>17</v>
       </c>
       <c r="D2" t="str">
-        <v>ABC123</v>
+        <v>9mm</v>
       </c>
       <c r="E2" t="str">
-        <v>9mm</v>
+        <v>ABC123456</v>
       </c>
       <c r="F2" t="str">
         <v>activo</v>
       </c>
       <c r="G2" t="str">
-        <v>empresa</v>
+        <v>PIST-001</v>
       </c>
       <c r="H2" t="str">
-        <v>01/01/2024</v>
+        <v>Puesto Central</v>
       </c>
       <c r="I2" t="str">
+        <v>TEN-001</v>
+      </c>
+      <c r="J2" t="str">
+        <v>31/12/2025</v>
+      </c>
+      <c r="K2" t="str">
+        <v>PORT-001</v>
+      </c>
+      <c r="L2" t="str">
+        <v>31/12/2025</v>
+      </c>
+      <c r="M2" t="str">
         <v/>
       </c>
-      <c r="J2" t="str">
-        <v>1234567890101</v>
+      <c r="N2" t="str">
+        <v>Arma asignada a puesto permanente</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>escopeta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Mossberg</v>
+      </c>
+      <c r="C3" t="str">
+        <v>500</v>
+      </c>
+      <c r="D3" t="str">
+        <v>12</v>
+      </c>
+      <c r="E3" t="str">
+        <v>XYZ789012</v>
+      </c>
+      <c r="F3" t="str">
+        <v>activo</v>
+      </c>
+      <c r="G3" t="str">
+        <v>ESCO-001</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Puesto Central</v>
+      </c>
+      <c r="I3" t="str">
+        <v>TEN-002</v>
+      </c>
+      <c r="J3" t="str">
+        <v>30/06/2026</v>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update employee template with correct column names and instructions
Corrects naming discrepancies between the template and backend for employee data import, including salary, payment method, and position.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 79364079-29fa-4649-b8e8-2e43a0b876bf
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A80"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -503,247 +503,292 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
+        <v>COLABORADORES — columnas clave:</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
+        <v xml:space="preserve">  puesto_operativo : nombre EXACTO del puesto (igual que en hoja PUESTOS)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+        <v xml:space="preserve">  sueldo_base      : salario mensual en quetzales (ej: 3500)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
+        <v xml:space="preserve">  bonificacion_incentivo : bonificación mensual (ej: 250)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v xml:space="preserve">  forma_pago       : mensual | quincenal | semanal | transferencia | cheque | efectivo</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
+        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
+        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v xml:space="preserve">  aplica_igss      : si | no</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
+        <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A80"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1442,7 +1487,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:V2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1453,16 +1498,19 @@
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
     <col min="9" max="9" width="25.83203125" customWidth="1"/>
-    <col min="10" max="10" width="35.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="28.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
-    <col min="16" max="16" width="10.83203125" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="30.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
     <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="8.83203125" customWidth="1"/>
+    <col min="19" max="19" width="28.83203125" customWidth="1"/>
+    <col min="20" max="20" width="20.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1482,7 +1530,7 @@
         <v>estado_civil</v>
       </c>
       <c r="F1" t="str">
-        <v>numero_igss</v>
+        <v>igss_numero</v>
       </c>
       <c r="G1" t="str">
         <v>nit</v>
@@ -1494,34 +1542,43 @@
         <v>correo</v>
       </c>
       <c r="J1" t="str">
-        <v>direccion</v>
+        <v>sede</v>
       </c>
       <c r="K1" t="str">
-        <v>departamento</v>
+        <v>fecha_ingreso</v>
       </c>
       <c r="L1" t="str">
-        <v>municipio</v>
+        <v>tipo_personal</v>
       </c>
       <c r="M1" t="str">
-        <v>fecha_ingreso</v>
+        <v>estado_laboral</v>
       </c>
       <c r="N1" t="str">
-        <v>puesto_nombre</v>
+        <v>puesto_operativo</v>
       </c>
       <c r="O1" t="str">
-        <v>turno_nombre</v>
+        <v>sueldo_base</v>
       </c>
       <c r="P1" t="str">
-        <v>salario</v>
+        <v>bonificacion_incentivo</v>
       </c>
       <c r="Q1" t="str">
-        <v>bonificacion</v>
+        <v>forma_pago</v>
       </c>
       <c r="R1" t="str">
-        <v>tipo_pago</v>
+        <v>aplica_igss</v>
       </c>
       <c r="S1" t="str">
-        <v>activo</v>
+        <v>estado_igss</v>
+      </c>
+      <c r="T1" t="str">
+        <v>banco</v>
+      </c>
+      <c r="U1" t="str">
+        <v>cuenta_bancaria</v>
+      </c>
+      <c r="V1" t="str">
+        <v>notas</v>
       </c>
     </row>
     <row r="2">
@@ -1553,39 +1610,48 @@
         <v>jgarcia@isp.gt</v>
       </c>
       <c r="J2" t="str">
-        <v>5a Avenida 1-23 Zona 1</v>
+        <v>Guatemala</v>
       </c>
       <c r="K2" t="str">
-        <v>Guatemala</v>
+        <v>15/01/2024</v>
       </c>
       <c r="L2" t="str">
-        <v>Guatemala Ciudad</v>
+        <v>guardia</v>
       </c>
       <c r="M2" t="str">
-        <v>15/01/2024</v>
+        <v>activo</v>
       </c>
       <c r="N2" t="str">
         <v>Puesto Central</v>
       </c>
       <c r="O2" t="str">
-        <v>Turno Diurno 8h</v>
+        <v>3500</v>
       </c>
       <c r="P2" t="str">
-        <v>3500</v>
+        <v>250</v>
       </c>
       <c r="Q2" t="str">
-        <v>250</v>
+        <v>mensual</v>
       </c>
       <c r="R2" t="str">
-        <v>mensual</v>
+        <v>si</v>
       </c>
       <c r="S2" t="str">
-        <v>si</v>
+        <v>activo</v>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update template to reflect correct payment account types
Modify `generate-template.mjs` and `ISP_PlantillaMaestra_CargaInicial.xlsx` to use "Monetaria" or "Ahorro" for the `forma_pago` column, indicating bank account type instead of payment frequency.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: afdc337f-a6f8-49ae-bbf3-e058725ae982
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -523,7 +523,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  forma_pago       : mensual | quincenal | semanal | transferencia | cheque | efectivo</v>
+        <v xml:space="preserve">  forma_pago       : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
       </c>
     </row>
     <row r="26">
@@ -1631,7 +1631,7 @@
         <v>250</v>
       </c>
       <c r="Q2" t="str">
-        <v>mensual</v>
+        <v>Monetaria</v>
       </c>
       <c r="R2" t="str">
         <v>si</v>

</xml_diff>

<commit_message>
Update payment and banking information fields
Add a new `tipo_cuenta` field to store bank account type, and separate `forma_pago` to specify payment method (transfer, check, cash). This change impacts database schema, API routes, template generation, and front-end forms.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8612dc34-337b-467f-8ba8-a1cf133b5f86
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A80"/>
+  <dimension ref="A1:A81"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -523,272 +523,277 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  forma_pago       : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
+        <v xml:space="preserve">  forma_pago       : transferencia | cheque | efectivo   (cómo recibe su pago)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
+        <v xml:space="preserve">  tipo_cuenta      : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
+        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  aplica_igss      : si | no</v>
+        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v xml:space="preserve">  aplica_igss      : si | no</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
         <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A81"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1487,7 +1492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:W2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1505,12 +1510,13 @@
     <col min="14" max="14" width="30.83203125" customWidth="1"/>
     <col min="15" max="15" width="12.83203125" customWidth="1"/>
     <col min="16" max="16" width="22.83203125" customWidth="1"/>
-    <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="28.83203125" customWidth="1"/>
-    <col min="20" max="20" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="16.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="28.83203125" customWidth="1"/>
     <col min="21" max="21" width="20.83203125" customWidth="1"/>
-    <col min="22" max="22" width="30.83203125" customWidth="1"/>
+    <col min="22" max="22" width="20.83203125" customWidth="1"/>
+    <col min="23" max="23" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1566,18 +1572,21 @@
         <v>forma_pago</v>
       </c>
       <c r="R1" t="str">
+        <v>tipo_cuenta</v>
+      </c>
+      <c r="S1" t="str">
         <v>aplica_igss</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>estado_igss</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>banco</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>cuenta_bancaria</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>notas</v>
       </c>
     </row>
@@ -1631,27 +1640,30 @@
         <v>250</v>
       </c>
       <c r="Q2" t="str">
+        <v>transferencia</v>
+      </c>
+      <c r="R2" t="str">
         <v>Monetaria</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v>si</v>
       </c>
-      <c r="S2" t="str">
+      <c r="T2" t="str">
         <v>activo</v>
       </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
       <c r="U2" t="str">
-        <v/>
+        <v>Banrural</v>
       </c>
       <c r="V2" t="str">
+        <v>000-123456-0</v>
+      </c>
+      <c r="W2" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update master data template with new fields and instructions
Adds new columns to CLIENTES, PUESTOS, and COLABORADORES sheets, updates import logic for IGSS and position-related fields, and enhances instructions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bcb4aec9-b4e2-428f-9573-19675282bbde
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A81"/>
+  <dimension ref="A1:A96"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -513,287 +513,352 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  sueldo_base      : salario mensual en quetzales (ej: 3500)</v>
+        <v xml:space="preserve">  tipo_jornada     : completa | parcial | mixta  — IMPORTANTE para cálculo de planilla</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  bonificacion_incentivo : bonificación mensual (ej: 250)</v>
+        <v xml:space="preserve">  dia_descanso     : lunes | martes | miercoles | jueves | viernes | sabado | domingo</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  forma_pago       : transferencia | cheque | efectivo   (cómo recibe su pago)</v>
+        <v xml:space="preserve">  horas_contrato   : horas diarias según contrato (ej: 8, 12, 24)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  tipo_cuenta      : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
+        <v xml:space="preserve">  sueldo_base      : salario mensual en quetzales (ej: 3500)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
+        <v xml:space="preserve">  bonificacion_incentivo : bonificación incentivo mensual (ej: 250)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
+        <v xml:space="preserve">  bonificacion_1/2/3 : bonificaciones adicionales en Q — dejar vacío si no aplica</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  aplica_igss      : si | no</v>
+        <v xml:space="preserve">  limite_anticipo  : monto máximo de anticipo en Q — dejar vacío para sin límite</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
+        <v xml:space="preserve">  forma_pago       : transferencia | cheque | efectivo   (cómo recibe su pago)</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v xml:space="preserve">  tipo_cuenta      : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
+        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
+        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+        <v xml:space="preserve">  aplica_igss      : si | no   — CRÍTICO: el puesto también debe tener aplica_igss=si</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
+        <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
+        <v>PUESTOS — columnas clave:</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
+        <v xml:space="preserve">  aplica_igss  : si | no  — CRÍTICO PARA PLANILLA: si es 'no' el empleado NO tendrá IGSS</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v xml:space="preserve">                 aunque el empleado lo tenga activo. AMBOS deben ser 'si'.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
+        <v xml:space="preserve">  regimen_igss : IVS | EPS | EPS_IVS | no_aplica  (si aplica_igss=si, usar IVS)</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v xml:space="preserve">  salario_puesto : referencia salarial del puesto (opcional, para reportes y comparativas)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v xml:space="preserve">  tarifa_puesto  : tarifa de facturación mensual al cliente por este puesto (para comercial)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v>CLIENTES — columna nueva:</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  tarifa_base_mensual : monto mensual que paga el cliente en Q (para módulo comercial)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A96"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1180,24 +1245,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" customWidth="1"/>
     <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
-    <col min="16" max="16" width="30.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
+    <col min="16" max="16" width="25.83203125" customWidth="1"/>
+    <col min="17" max="17" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1217,36 +1283,39 @@
         <v>fecha_inicio_contrato</v>
       </c>
       <c r="F1" t="str">
+        <v>tarifa_base_mensual</v>
+      </c>
+      <c r="G1" t="str">
         <v>igss_aplica</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>igss_codigo_centro</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>igss_direccion</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>igss_zona</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>igss_departamento</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>igss_municipio</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>igss_codigo_actividad</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>igss_contacto</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>igss_telefono</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>igss_email</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>notas</v>
       </c>
     </row>
@@ -1267,16 +1336,16 @@
         <v>15/01/2024</v>
       </c>
       <c r="F2" t="str">
+        <v>15000</v>
+      </c>
+      <c r="G2" t="str">
         <v>si</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>01</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>5a Calle 5-50</v>
-      </c>
-      <c r="I2" t="str">
-        <v>1</v>
       </c>
       <c r="J2" t="str">
         <v>1</v>
@@ -1285,24 +1354,27 @@
         <v>1</v>
       </c>
       <c r="L2" t="str">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
         <v>0851</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Juan Pérez</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>55551234</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>igss@ejemplo.com</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1417,12 +1489,12 @@
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1436,22 +1508,22 @@
         <v>turno_nombre</v>
       </c>
       <c r="D1" t="str">
-        <v>codigo</v>
+        <v>ubicacion</v>
       </c>
       <c r="E1" t="str">
-        <v>ubicacion</v>
+        <v>aplica_igss</v>
       </c>
       <c r="F1" t="str">
+        <v>regimen_igss</v>
+      </c>
+      <c r="G1" t="str">
+        <v>salario_puesto</v>
+      </c>
+      <c r="H1" t="str">
+        <v>tarifa_puesto</v>
+      </c>
+      <c r="I1" t="str">
         <v>descripcion</v>
-      </c>
-      <c r="G1" t="str">
-        <v>salario_base</v>
-      </c>
-      <c r="H1" t="str">
-        <v>num_guardias_requeridos</v>
-      </c>
-      <c r="I1" t="str">
-        <v>activo</v>
       </c>
     </row>
     <row r="2">
@@ -1465,22 +1537,22 @@
         <v>Turno Diurno 8h</v>
       </c>
       <c r="D2" t="str">
-        <v>P-001</v>
+        <v>Zona 10 Recepción</v>
       </c>
       <c r="E2" t="str">
-        <v>Zona 10</v>
+        <v>si</v>
       </c>
       <c r="F2" t="str">
+        <v>IVS</v>
+      </c>
+      <c r="G2" t="str">
+        <v>3200</v>
+      </c>
+      <c r="H2" t="str">
+        <v>5500</v>
+      </c>
+      <c r="I2" t="str">
         <v>Recepción principal</v>
-      </c>
-      <c r="G2" t="str">
-        <v>3500</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2</v>
-      </c>
-      <c r="I2" t="str">
-        <v>si</v>
       </c>
     </row>
   </sheetData>
@@ -1492,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:AE2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1502,21 +1574,29 @@
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="15.83203125" customWidth="1"/>
-    <col min="14" max="14" width="30.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="22.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="15.83203125" customWidth="1"/>
+    <col min="15" max="15" width="30.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
     <col min="18" max="18" width="14.83203125" customWidth="1"/>
     <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="28.83203125" customWidth="1"/>
-    <col min="21" max="21" width="20.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
-    <col min="23" max="23" width="30.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
+    <col min="23" max="23" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="25" max="25" width="16.83203125" customWidth="1"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1"/>
+    <col min="27" max="27" width="12.83203125" customWidth="1"/>
+    <col min="28" max="28" width="28.83203125" customWidth="1"/>
+    <col min="29" max="29" width="20.83203125" customWidth="1"/>
+    <col min="30" max="30" width="20.83203125" customWidth="1"/>
+    <col min="31" max="31" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1545,48 +1625,72 @@
         <v>telefono</v>
       </c>
       <c r="I1" t="str">
+        <v>telefono_secundario</v>
+      </c>
+      <c r="J1" t="str">
         <v>correo</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>sede</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>fecha_ingreso</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>tipo_personal</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>estado_laboral</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>puesto_operativo</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
+        <v>tipo_jornada</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>dia_descanso</v>
+      </c>
+      <c r="R1" t="str">
+        <v>horas_contrato</v>
+      </c>
+      <c r="S1" t="str">
         <v>sueldo_base</v>
       </c>
-      <c r="P1" t="str">
+      <c r="T1" t="str">
         <v>bonificacion_incentivo</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="U1" t="str">
+        <v>bonificacion_1</v>
+      </c>
+      <c r="V1" t="str">
+        <v>bonificacion_2</v>
+      </c>
+      <c r="W1" t="str">
+        <v>bonificacion_3</v>
+      </c>
+      <c r="X1" t="str">
+        <v>limite_anticipo</v>
+      </c>
+      <c r="Y1" t="str">
         <v>forma_pago</v>
       </c>
-      <c r="R1" t="str">
+      <c r="Z1" t="str">
         <v>tipo_cuenta</v>
       </c>
-      <c r="S1" t="str">
+      <c r="AA1" t="str">
         <v>aplica_igss</v>
       </c>
-      <c r="T1" t="str">
+      <c r="AB1" t="str">
         <v>estado_igss</v>
       </c>
-      <c r="U1" t="str">
+      <c r="AC1" t="str">
         <v>banco</v>
       </c>
-      <c r="V1" t="str">
+      <c r="AD1" t="str">
         <v>cuenta_bancaria</v>
       </c>
-      <c r="W1" t="str">
+      <c r="AE1" t="str">
         <v>notas</v>
       </c>
     </row>
@@ -1616,54 +1720,78 @@
         <v>55551234</v>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>jgarcia@isp.gt</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Guatemala</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>15/01/2024</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>guardia</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>activo</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>Puesto Central</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
+        <v>completa</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>domingo</v>
+      </c>
+      <c r="R2" t="str">
+        <v>8</v>
+      </c>
+      <c r="S2" t="str">
         <v>3500</v>
       </c>
-      <c r="P2" t="str">
+      <c r="T2" t="str">
         <v>250</v>
       </c>
-      <c r="Q2" t="str">
-        <v>transferencia</v>
-      </c>
-      <c r="R2" t="str">
-        <v>Monetaria</v>
-      </c>
-      <c r="S2" t="str">
-        <v>si</v>
-      </c>
-      <c r="T2" t="str">
-        <v>activo</v>
-      </c>
       <c r="U2" t="str">
-        <v>Banrural</v>
+        <v/>
       </c>
       <c r="V2" t="str">
-        <v>000-123456-0</v>
+        <v/>
       </c>
       <c r="W2" t="str">
         <v/>
       </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v>transferencia</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Monetaria</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>si</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>activo</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Banrural</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>000-123456-0</v>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new sheets for client branches and supervision areas
Add SEDES and ZONAS sheets to the template, update PUESTOS with new columns, and adjust import logic and order.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 622cd329-d539-4a32-a643-5a2afc166612
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -6,18 +6,20 @@
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
     <sheet name="CLIENTES" sheetId="2" r:id="rId2"/>
     <sheet name="TURNOS" sheetId="3" r:id="rId3"/>
-    <sheet name="PUESTOS" sheetId="4" r:id="rId4"/>
-    <sheet name="COLABORADORES" sheetId="5" r:id="rId5"/>
-    <sheet name="ARMAS" sheetId="6" r:id="rId6"/>
-    <sheet name="VEHICULOS" sheetId="7" r:id="rId7"/>
-    <sheet name="BODEGA_CATEGORIAS" sheetId="8" r:id="rId8"/>
-    <sheet name="BODEGA_ARTICULOS" sheetId="9" r:id="rId9"/>
-    <sheet name="ANTICIPOS" sheetId="10" r:id="rId10"/>
-    <sheet name="HISTORIAL_PRESTACIONES" sheetId="11" r:id="rId11"/>
-    <sheet name="USUARIOS" sheetId="12" r:id="rId12"/>
-    <sheet name="ROLES" sheetId="13" r:id="rId13"/>
-    <sheet name="MODULOS" sheetId="14" r:id="rId14"/>
-    <sheet name="IGSS_PATRONO" sheetId="15" r:id="rId15"/>
+    <sheet name="SEDES" sheetId="4" r:id="rId4"/>
+    <sheet name="PUESTOS" sheetId="5" r:id="rId5"/>
+    <sheet name="COLABORADORES" sheetId="6" r:id="rId6"/>
+    <sheet name="ZONAS" sheetId="7" r:id="rId7"/>
+    <sheet name="ARMAS" sheetId="8" r:id="rId8"/>
+    <sheet name="VEHICULOS" sheetId="9" r:id="rId9"/>
+    <sheet name="BODEGA_CATEGORIAS" sheetId="10" r:id="rId10"/>
+    <sheet name="BODEGA_ARTICULOS" sheetId="11" r:id="rId11"/>
+    <sheet name="ANTICIPOS" sheetId="12" r:id="rId12"/>
+    <sheet name="HISTORIAL_PRESTACIONES" sheetId="13" r:id="rId13"/>
+    <sheet name="USUARIOS" sheetId="14" r:id="rId14"/>
+    <sheet name="ROLES" sheetId="15" r:id="rId15"/>
+    <sheet name="MODULOS" sheetId="16" r:id="rId16"/>
+    <sheet name="IGSS_PATRONO" sheetId="17" r:id="rId17"/>
   </sheets>
 </workbook>
 </file>
@@ -411,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A96"/>
+  <dimension ref="A1:A110"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -438,432 +440,596 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. PUESTOS</v>
+        <v>3. SEDES        (sucursales de clientes — depende de CLIENTES)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>4. COLABORADORES</v>
+        <v>4. PUESTOS      (depende de CLIENTES, TURNOS y SEDES)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5. ARMAS</v>
+        <v>5. COLABORADORES (depende de PUESTOS)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6. VEHICULOS</v>
+        <v>6. ZONAS        (áreas de supervisión — depende de COLABORADORES para el supervisor)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>7. BODEGA_CATEGORIAS</v>
+        <v>7. ARMAS</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>8. BODEGA_ARTICULOS</v>
+        <v>8. VEHICULOS</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>9. ANTICIPOS</v>
+        <v>9. BODEGA_CATEGORIAS</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>10. HISTORIAL_PRESTACIONES</v>
+        <v>10. BODEGA_ARTICULOS</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>11. USUARIOS</v>
+        <v>11. ANTICIPOS</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>12. ROLES</v>
+        <v>12. HISTORIAL_PRESTACIONES</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>13. MODULOS</v>
+        <v>13. USUARIOS</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>14. IGSS_PATRONO</v>
+        <v>14. ROLES</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>15. MODULOS</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>FORMATO DE FECHAS: dd/mm/aaaa   Ejemplo: 15/01/2024</v>
+        <v>16. IGSS_PATRONO</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>COLABORADORES — columnas clave:</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v xml:space="preserve">  puesto_operativo : nombre EXACTO del puesto (igual que en hoja PUESTOS)</v>
+        <v>FORMATO DE FECHAS: dd/mm/aaaa   Ejemplo: 15/01/2024</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  tipo_jornada     : completa | parcial | mixta  — IMPORTANTE para cálculo de planilla</v>
+        <v>COLABORADORES — columnas clave:</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  dia_descanso     : lunes | martes | miercoles | jueves | viernes | sabado | domingo</v>
+        <v xml:space="preserve">  puesto_operativo : nombre EXACTO del puesto (igual que en hoja PUESTOS)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  horas_contrato   : horas diarias según contrato (ej: 8, 12, 24)</v>
+        <v xml:space="preserve">  tipo_jornada     : completa | parcial | mixta  — IMPORTANTE para cálculo de planilla</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  sueldo_base      : salario mensual en quetzales (ej: 3500)</v>
+        <v xml:space="preserve">  dia_descanso     : lunes | martes | miercoles | jueves | viernes | sabado | domingo</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  bonificacion_incentivo : bonificación incentivo mensual (ej: 250)</v>
+        <v xml:space="preserve">  horas_contrato   : horas diarias según contrato (ej: 8, 12, 24)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  bonificacion_1/2/3 : bonificaciones adicionales en Q — dejar vacío si no aplica</v>
+        <v xml:space="preserve">  sueldo_base      : salario mensual en quetzales (ej: 3500)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  limite_anticipo  : monto máximo de anticipo en Q — dejar vacío para sin límite</v>
+        <v xml:space="preserve">  bonificacion_incentivo : bonificación incentivo mensual (ej: 250)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  forma_pago       : transferencia | cheque | efectivo   (cómo recibe su pago)</v>
+        <v xml:space="preserve">  bonificacion_1/2/3 : bonificaciones adicionales en Q — dejar vacío si no aplica</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  tipo_cuenta      : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
+        <v xml:space="preserve">  limite_anticipo  : monto máximo de anticipo en Q — dejar vacío para sin límite</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
+        <v xml:space="preserve">  forma_pago       : transferencia | cheque | efectivo   (cómo recibe su pago)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
+        <v xml:space="preserve">  tipo_cuenta      : Monetaria | Ahorro   (tipo de cuenta bancaria, puede quedar vacío)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">  aplica_igss      : si | no   — CRÍTICO: el puesto también debe tener aplica_igss=si</v>
+        <v xml:space="preserve">  tipo_personal    : guardia | supervisor | jefe_servicio | administrativo_bodega | administrativo_rrhh | gerencia</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
+        <v xml:space="preserve">  estado_laboral   : activo | suspendido | baja | licencia</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">  aplica_igss      : si | no   — CRÍTICO: el puesto también debe tener aplica_igss=si</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PUESTOS — columnas clave:</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v xml:space="preserve">  aplica_igss  : si | no  — CRÍTICO PARA PLANILLA: si es 'no' el empleado NO tendrá IGSS</v>
+        <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">                 aunque el empleado lo tenga activo. AMBOS deben ser 'si'.</v>
+        <v>PUESTOS — columnas clave:</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  regimen_igss : IVS | EPS | EPS_IVS | no_aplica  (si aplica_igss=si, usar IVS)</v>
+        <v xml:space="preserve">  aplica_igss  : si | no  — CRÍTICO PARA PLANILLA: si es 'no' el empleado NO tendrá IGSS</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">  salario_puesto : referencia salarial del puesto (opcional, para reportes y comparativas)</v>
+        <v xml:space="preserve">                 aunque el empleado lo tenga activo. AMBOS deben ser 'si'.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v xml:space="preserve">  tarifa_puesto  : tarifa de facturación mensual al cliente por este puesto (para comercial)</v>
+        <v xml:space="preserve">  regimen_igss : IVS | EPS | EPS_IVS | no_aplica  (si aplica_igss=si, usar IVS)</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  salario_puesto : referencia salarial del puesto (opcional, para reportes y comparativas)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v xml:space="preserve">  tarifa_puesto  : tarifa de facturación mensual al cliente por este puesto (para comercial)</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>CLIENTES — columna nueva:</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v xml:space="preserve">  tarifa_base_mensual : monto mensual que paga el cliente en Q (para módulo comercial)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
+        <v xml:space="preserve">  tarifa_base_mensual : monto mensual que paga el cliente en Q (para módulo comercial)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+        <v>SEDES — columnas clave:</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
+        <v xml:space="preserve">  cliente_nombre : nombre EXACTO del cliente (igual que en hoja CLIENTES)</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v xml:space="preserve">  nombre         : nombre de la sede/sucursal (ej: Sede Central, Bodega Norte)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
+        <v xml:space="preserve">  ciudad         : ciudad donde está la sede</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v>ZONAS — columnas clave:</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
+        <v xml:space="preserve">  nombre          : nombre del área de supervisión (ej: Zona Norte, Zona Sur)</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v xml:space="preserve">  descripcion     : descripción breve del área</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
+        <v xml:space="preserve">  supervisor_dpi  : DPI del colaborador supervisor de la zona (de hoja COLABORADORES)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
+        <v xml:space="preserve">  NOTA: el pizarrón agrupa los puestos por zona. Si un puesto no tiene zona,</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
+        <v xml:space="preserve">  aparecerá en 'Sin zona' en el pizarrón.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A96"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A110"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>descripcion</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Uniformes</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Ropa y equipo personal</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="35.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>categoria_nombre</v>
+      </c>
+      <c r="C1" t="str">
+        <v>codigo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>unidad_medida</v>
+      </c>
+      <c r="E1" t="str">
+        <v>stock_actual</v>
+      </c>
+      <c r="F1" t="str">
+        <v>stock_minimo</v>
+      </c>
+      <c r="G1" t="str">
+        <v>precio_unitario</v>
+      </c>
+      <c r="H1" t="str">
+        <v>descripcion</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Camisa negra talla M</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Uniformes</v>
+      </c>
+      <c r="C2" t="str">
+        <v>UNI-CAM-M</v>
+      </c>
+      <c r="D2" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="E2" t="str">
+        <v>50</v>
+      </c>
+      <c r="F2" t="str">
+        <v>10</v>
+      </c>
+      <c r="G2" t="str">
+        <v>85</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <cols>
@@ -915,7 +1081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G2"/>
   <cols>
@@ -981,7 +1147,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J2"/>
   <cols>
@@ -1068,7 +1234,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <cols>
@@ -1120,7 +1286,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5"/>
   <cols>
@@ -1191,7 +1357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <cols>
@@ -1484,7 +1650,96 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:G3"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>cliente_nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="C1" t="str">
+        <v>direccion</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ciudad</v>
+      </c>
+      <c r="E1" t="str">
+        <v>contacto</v>
+      </c>
+      <c r="F1" t="str">
+        <v>telefono</v>
+      </c>
+      <c r="G1" t="str">
+        <v>notas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Comercializadora Ejemplo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Sede Central</v>
+      </c>
+      <c r="C2" t="str">
+        <v>5a Calle 5-50 Zona 10</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Guatemala</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Carlos López</v>
+      </c>
+      <c r="F2" t="str">
+        <v>55551234</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Comercializadora Ejemplo</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bodega Norte</v>
+      </c>
+      <c r="C3" t="str">
+        <v>12 Av. 8-20 Zona 2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Guatemala</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Ana Pérez</v>
+      </c>
+      <c r="F3" t="str">
+        <v>55559876</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1492,9 +1747,11 @@
     <col min="4" max="4" width="25.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="35.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1517,12 +1774,18 @@
         <v>regimen_igss</v>
       </c>
       <c r="G1" t="str">
+        <v>zona_nombre</v>
+      </c>
+      <c r="H1" t="str">
+        <v>sede_nombre</v>
+      </c>
+      <c r="I1" t="str">
         <v>salario_puesto</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>tarifa_puesto</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>descripcion</v>
       </c>
     </row>
@@ -1546,23 +1809,29 @@
         <v>IVS</v>
       </c>
       <c r="G2" t="str">
+        <v>Zona Sur</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Sede Central</v>
+      </c>
+      <c r="I2" t="str">
         <v>3200</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>5500</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Recepción principal</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AE2"/>
   <cols>
@@ -1796,7 +2065,67 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="50.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>descripcion</v>
+      </c>
+      <c r="C1" t="str">
+        <v>supervisor_dpi</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Zona Norte</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Puestos en zona norte de la ciudad — clientes industriales</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Zona Sur</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Puestos en zona sur — centros comerciales y oficinas</v>
+      </c>
+      <c r="C3" t="str">
+        <v>9876543210101</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Zona Oriente</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Clientes en carretera al atlántico</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N3"/>
   <cols>
@@ -1955,7 +2284,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J2"/>
   <cols>
@@ -2040,108 +2369,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>nombre</v>
-      </c>
-      <c r="B1" t="str">
-        <v>descripcion</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Uniformes</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Ropa y equipo personal</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="35.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>nombre</v>
-      </c>
-      <c r="B1" t="str">
-        <v>categoria_nombre</v>
-      </c>
-      <c r="C1" t="str">
-        <v>codigo</v>
-      </c>
-      <c r="D1" t="str">
-        <v>unidad_medida</v>
-      </c>
-      <c r="E1" t="str">
-        <v>stock_actual</v>
-      </c>
-      <c r="F1" t="str">
-        <v>stock_minimo</v>
-      </c>
-      <c r="G1" t="str">
-        <v>precio_unitario</v>
-      </c>
-      <c r="H1" t="str">
-        <v>descripcion</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Camisa negra talla M</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Uniformes</v>
-      </c>
-      <c r="C2" t="str">
-        <v>UNI-CAM-M</v>
-      </c>
-      <c r="D2" t="str">
-        <v>unidad</v>
-      </c>
-      <c r="E2" t="str">
-        <v>50</v>
-      </c>
-      <c r="F2" t="str">
-        <v>10</v>
-      </c>
-      <c r="G2" t="str">
-        <v>85</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add essential details for shift scheduling and employee assignments
Update import logic to include shift start dates and times, employee order for shifts, and automatically generate work/rest slots based on shift types.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 439cf89a-ae13-4a85-85a4-05838cb94dd5
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/artifacts/isp-web/public/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A110"/>
+  <dimension ref="A1:A118"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -588,339 +588,379 @@
         <v xml:space="preserve">  estado_igss      : activo | no_activo | pendiente_regularizacion</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">  orden_titular    : 1 o 2 — CRÍTICO PIZARRÓN para turnos 24x24</v>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PUESTOS — columnas clave:</v>
+        <v xml:space="preserve">                     orden 1 = trabaja días impares del ciclo (1,3,5,7,9,11,13)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">  aplica_igss  : si | no  — CRÍTICO PARA PLANILLA: si es 'no' el empleado NO tendrá IGSS</v>
+        <v xml:space="preserve">                     orden 2 = trabaja días pares del ciclo (2,4,6,8,10,12,14)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v xml:space="preserve">                 aunque el empleado lo tenga activo. AMBOS deben ser 'si'.</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v xml:space="preserve">  regimen_igss : IVS | EPS | EPS_IVS | no_aplica  (si aplica_igss=si, usar IVS)</v>
+        <v xml:space="preserve">                     Si hay un solo guardia por puesto, dejar en 1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v xml:space="preserve">  salario_puesto : referencia salarial del puesto (opcional, para reportes y comparativas)</v>
+        <v>PUESTOS — columnas clave:</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v xml:space="preserve">  tarifa_puesto  : tarifa de facturación mensual al cliente por este puesto (para comercial)</v>
+        <v xml:space="preserve">  aplica_igss      : si | no  — CRÍTICO PARA PLANILLA: si es 'no' el empleado NO tendrá IGSS</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v xml:space="preserve">                     aunque el empleado lo tenga activo. AMBOS deben ser 'si'.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>CLIENTES — columna nueva:</v>
+        <v xml:space="preserve">  regimen_igss     : IVS | EPS | EPS_IVS | no_aplica  (si aplica_igss=si, usar IVS)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v xml:space="preserve">  tarifa_base_mensual : monto mensual que paga el cliente en Q (para módulo comercial)</v>
+        <v xml:space="preserve">  fecha_inicio_ciclo : CRÍTICO PIZARRÓN: fecha ancla del ciclo de turnos (dd/mm/aaaa)</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v xml:space="preserve">                     Usa el primer día que ese puesto arrancó con el turno actual.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SEDES — columnas clave:</v>
+        <v xml:space="preserve">                     Sin esta fecha el pizarrón no sabe qué día del ciclo es hoy.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v xml:space="preserve">  cliente_nombre : nombre EXACTO del cliente (igual que en hoja CLIENTES)</v>
+        <v xml:space="preserve">  hora_entrada     : hora de inicio de turno en formato HH:MM (ej: 07:00, 19:00, 06:00)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v xml:space="preserve">  nombre         : nombre de la sede/sucursal (ej: Sede Central, Bodega Norte)</v>
+        <v xml:space="preserve">  salario_puesto   : referencia salarial del puesto (opcional, para reportes y comparativas)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v xml:space="preserve">  ciudad         : ciudad donde está la sede</v>
+        <v xml:space="preserve">  tarifa_puesto    : tarifa de facturación mensual al cliente por este puesto (para comercial)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ZONAS — columnas clave:</v>
+        <v>CLIENTES — columna nueva:</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v xml:space="preserve">  nombre          : nombre del área de supervisión (ej: Zona Norte, Zona Sur)</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v xml:space="preserve">  descripcion     : descripción breve del área</v>
+        <v xml:space="preserve">  tarifa_base_mensual : monto mensual que paga el cliente en Q (para módulo comercial)</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v xml:space="preserve">  supervisor_dpi  : DPI del colaborador supervisor de la zona (de hoja COLABORADORES)</v>
+        <v>SEDES — columnas clave:</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v xml:space="preserve">  NOTA: el pizarrón agrupa los puestos por zona. Si un puesto no tiene zona,</v>
+        <v xml:space="preserve">  cliente_nombre : nombre EXACTO del cliente (igual que en hoja CLIENTES)</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v xml:space="preserve">  aparecerá en 'Sin zona' en el pizarrón.</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
+        <v xml:space="preserve">  nombre         : nombre de la sede/sucursal (ej: Sede Central, Bodega Norte)</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v xml:space="preserve">  ciudad         : ciudad donde está la sede</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
+        <v>ZONAS — columnas clave:</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
+        <v xml:space="preserve">  nombre          : nombre del área de supervisión (ej: Zona Norte, Zona Sur)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
+        <v xml:space="preserve">  descripcion     : descripción breve del área</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v xml:space="preserve">  supervisor_dpi  : DPI del colaborador supervisor de la zona (de hoja COLABORADORES)</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
+        <v xml:space="preserve">  NOTA: el pizarrón agrupa los puestos por zona. Si un puesto no tiene zona,</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
+        <v xml:space="preserve">  aparecerá en 'Sin zona' en el pizarrón.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
+        <v>ARMAS — El arma se asigna al PUESTO (puesto_nombre), NO al empleado.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v xml:space="preserve">  El campo custodio_dpi es opcional: solo si quieres registrar quién la tiene HOY.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
+        <v xml:space="preserve">  Los agentes que trabajan el puesto son responsables del arma durante su turno.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="str">
-        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
+        <v xml:space="preserve">  codigo: si se deja vacío, el sistema genera uno automático (PIST-001, ESCO-001...).</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
+        <v>TURNOS — columnas: nombre | horas_trabajo | horas_descanso | num_titulares | descripcion</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 24x24: horas_trabajo=24, horas_descanso=24, descripcion="07:00 a 07:00 del día siguiente"</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 12x12: horas_trabajo=12, horas_descanso=12</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="str">
-        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
+        <v xml:space="preserve">  Turno 8h   : horas_trabajo=8,  horas_descanso=16</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
+        <v>MÓDULOS VÁLIDOS (columnas modulos en ROLES / modulo_clave en MODULOS):</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  dashboard  →  Dashboard  (General)</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  pizarron  →  Pizarrón Operativo  (Operaciones)</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  seguimiento_ssa  →  Seguimiento SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
+        <v xml:space="preserve">  pipeline_ssa  →  Pipeline SSA  (Operaciones)</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  tareas  →  Tareas  (Operaciones)</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  incidencias  →  Incidencias  (Operaciones)</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  custodias  →  Custodias  (Operaciones)</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  cambios_estructurales  →  Cambios Estructurales  (Operaciones)</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  clientes  →  Clientes  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  comercial  →  Comercial  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reportes  →  Reportería  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  kpi  →  KPI &amp; Métricas  (Clientes &amp; Comercial)</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  empleados  →  Colaboradores  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  reclutamiento  →  Reclutamiento  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  anticipos  →  Anticipos  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  eventos_rrhh  →  Eventos RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  alertas_rrhh  →  Alertas RRHH  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  nomina  →  Novedades de Nómina  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  pre_planilla  →  Pre-Planilla  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  planilla  →  Planilla Final  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
+        <v xml:space="preserve">  turnos  →  Tipos de Turno  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
+        <v xml:space="preserve">  cambios_salariales  →  Cambios Salariales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+        <v xml:space="preserve">  prestaciones  →  Prestaciones Laborales  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  solicitudes_vacaciones  →  Solicitudes de Vacaciones  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+        <v xml:space="preserve">  planillas_especiales  →  Bono 14 &amp; Aguinaldo  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+        <v xml:space="preserve">  libro_salarios  →  Libro de Salarios  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  igss_planilla  →  Planilla IGSS  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  carnets_qr  →  Carnets QR  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+        <v xml:space="preserve">  kiosco_solicitudes  →  Solicitudes Kiosco  (Personal &amp; RRHH)</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+        <v xml:space="preserve">  solicitudes_eliminacion  →  Solicitudes de Eliminación  (Sistema)</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
+        <v xml:space="preserve">  usuarios  →  Usuarios del Sistema  (Sistema)</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v xml:space="preserve">  config_whatsapp  →  Configuración WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v xml:space="preserve">  cms  →  CMS Web  (Sistema)</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v xml:space="preserve">  simulador_wa  →  Simulador WhatsApp  (Sistema)</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v xml:space="preserve">  bodega  →  Inventario General  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v xml:space="preserve">  vehiculos  →  Vehículos  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v xml:space="preserve">  armeria  →  Armería  (Bodega e Inventario)</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v xml:space="preserve">  importacion  →  Importar Datos  (Migración)</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
         <v xml:space="preserve">  control_qr  →  Control Operativo QR  (Control Operativo)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A118"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1739,7 +1779,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1749,9 +1789,11 @@
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="22.83203125" customWidth="1"/>
     <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1780,12 +1822,18 @@
         <v>sede_nombre</v>
       </c>
       <c r="I1" t="str">
+        <v>fecha_inicio_ciclo</v>
+      </c>
+      <c r="J1" t="str">
+        <v>hora_entrada</v>
+      </c>
+      <c r="K1" t="str">
         <v>salario_puesto</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>tarifa_puesto</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>descripcion</v>
       </c>
     </row>
@@ -1797,7 +1845,7 @@
         <v>Comercializadora Ejemplo</v>
       </c>
       <c r="C2" t="str">
-        <v>Turno Diurno 8h</v>
+        <v>Turno 24x24</v>
       </c>
       <c r="D2" t="str">
         <v>Zona 10 Recepción</v>
@@ -1815,25 +1863,31 @@
         <v>Sede Central</v>
       </c>
       <c r="I2" t="str">
+        <v>07/04/2025</v>
+      </c>
+      <c r="J2" t="str">
+        <v>07:00</v>
+      </c>
+      <c r="K2" t="str">
         <v>3200</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>5500</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>Recepción principal</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AF3"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -1853,19 +1907,20 @@
     <col min="16" max="16" width="14.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" customWidth="1"/>
     <col min="18" max="18" width="14.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
     <col min="25" max="25" width="16.83203125" customWidth="1"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="28" width="28.83203125" customWidth="1"/>
-    <col min="29" max="29" width="20.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1"/>
+    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="29" max="29" width="28.83203125" customWidth="1"/>
     <col min="30" max="30" width="20.83203125" customWidth="1"/>
-    <col min="31" max="31" width="30.83203125" customWidth="1"/>
+    <col min="31" max="31" width="20.83203125" customWidth="1"/>
+    <col min="32" max="32" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1915,51 +1970,54 @@
         <v>puesto_operativo</v>
       </c>
       <c r="P1" t="str">
+        <v>orden_titular</v>
+      </c>
+      <c r="Q1" t="str">
         <v>tipo_jornada</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>dia_descanso</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>horas_contrato</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>sueldo_base</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>bonificacion_incentivo</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>bonificacion_1</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>bonificacion_2</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>bonificacion_3</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>limite_anticipo</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>forma_pago</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>tipo_cuenta</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>aplica_igss</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>estado_igss</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>banco</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>cuenta_bancaria</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AF1" t="str">
         <v>notas</v>
       </c>
     </row>
@@ -2010,22 +2068,22 @@
         <v>Puesto Central</v>
       </c>
       <c r="P2" t="str">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="str">
         <v>completa</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>domingo</v>
       </c>
-      <c r="R2" t="str">
-        <v>8</v>
-      </c>
       <c r="S2" t="str">
+        <v>24</v>
+      </c>
+      <c r="T2" t="str">
         <v>3500</v>
       </c>
-      <c r="T2" t="str">
+      <c r="U2" t="str">
         <v>250</v>
-      </c>
-      <c r="U2" t="str">
-        <v/>
       </c>
       <c r="V2" t="str">
         <v/>
@@ -2037,30 +2095,131 @@
         <v/>
       </c>
       <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
         <v>transferencia</v>
       </c>
-      <c r="Z2" t="str">
+      <c r="AA2" t="str">
         <v>Monetaria</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AB2" t="str">
         <v>si</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AC2" t="str">
         <v>activo</v>
       </c>
-      <c r="AC2" t="str">
+      <c r="AD2" t="str">
         <v>Banrural</v>
       </c>
-      <c r="AD2" t="str">
+      <c r="AE2" t="str">
         <v>000-123456-0</v>
       </c>
-      <c r="AE2" t="str">
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>9876543210101</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Pedro Ajú Choc</v>
+      </c>
+      <c r="C3" t="str">
+        <v>10/11/1988</v>
+      </c>
+      <c r="D3" t="str">
+        <v>masculino</v>
+      </c>
+      <c r="E3" t="str">
+        <v>casado</v>
+      </c>
+      <c r="F3" t="str">
+        <v>87654321</v>
+      </c>
+      <c r="G3" t="str">
+        <v>7654321-0</v>
+      </c>
+      <c r="H3" t="str">
+        <v>55559876</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>paju@isp.gt</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Guatemala</v>
+      </c>
+      <c r="L3" t="str">
+        <v>15/01/2024</v>
+      </c>
+      <c r="M3" t="str">
+        <v>guardia</v>
+      </c>
+      <c r="N3" t="str">
+        <v>activo</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Puesto Central</v>
+      </c>
+      <c r="P3" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>completa</v>
+      </c>
+      <c r="R3" t="str">
+        <v>sabado</v>
+      </c>
+      <c r="S3" t="str">
+        <v>24</v>
+      </c>
+      <c r="T3" t="str">
+        <v>3500</v>
+      </c>
+      <c r="U3" t="str">
+        <v>250</v>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v>transferencia</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Monetaria</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>si</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>activo</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>Banrural</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>000-654321-0</v>
+      </c>
+      <c r="AF3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>